<commit_message>
Poging implementatie threads. Nog niet gelukt
</commit_message>
<xml_diff>
--- a/TODO.xlsx
+++ b/TODO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6BB675-1AB6-4B37-A836-CEA805BD88A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1D19B6-37A0-426D-B589-E83835A7BFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{453B4A97-9B0D-4640-BCE1-44769073F81C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="55">
   <si>
     <t>Belang</t>
   </si>
@@ -195,6 +195,15 @@
   </si>
   <si>
     <t xml:space="preserve">In de onderstaande lijst zijn globale mijlpalen toegevoegd. Dit zijn niet taken, maar punten op de horizon. </t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Zonder HR-database</t>
+  </si>
+  <si>
+    <t>(CMD) applicatie bruikbaar maken zonder HR-database</t>
   </si>
 </sst>
 </file>
@@ -267,6 +276,90 @@
   <dxfs count="22">
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -313,62 +406,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -419,6 +456,76 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -437,123 +544,25 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -611,36 +620,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}" name="Tabel13" displayName="Tabel13" ref="A3:H7" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A3:H7" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}" name="Tabel13" displayName="Tabel13" ref="A3:H8" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+  <autoFilter ref="A3:H8" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}"/>
   <tableColumns count="8">
-    <tableColumn id="11" xr3:uid="{03EDA042-17EA-4CE6-B062-BCF9D6DC876F}" name="Belang" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{463702E7-7165-4523-9D6B-7ACDA80B9EBD}" name="Prioriteit" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{54B6E275-8C75-4272-90E9-4F6FAD3E0236}" name="Naam" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{49D3B12A-D2A9-4E25-B74D-6BCBEBD88EFA}" name="Beschrijving" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{8FD3869D-6875-466A-8DF3-E625CE109EA2}" name="Application part" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{D973CD04-220F-4A8C-9BF5-59F7D87A76C1}" name="Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{C850139A-3749-435E-9416-B011E18BC87E}" name="Persoon" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{10DD826D-3BF7-4FA1-95A9-305EEE094144}" name="Opmerking" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{03EDA042-17EA-4CE6-B062-BCF9D6DC876F}" name="Belang" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{463702E7-7165-4523-9D6B-7ACDA80B9EBD}" name="Prioriteit" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{54B6E275-8C75-4272-90E9-4F6FAD3E0236}" name="Naam" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{49D3B12A-D2A9-4E25-B74D-6BCBEBD88EFA}" name="Beschrijving" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{8FD3869D-6875-466A-8DF3-E625CE109EA2}" name="Application part" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{D973CD04-220F-4A8C-9BF5-59F7D87A76C1}" name="Status" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{C850139A-3749-435E-9416-B011E18BC87E}" name="Persoon" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{10DD826D-3BF7-4FA1-95A9-305EEE094144}" name="Opmerking" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}" name="Tabel1" displayName="Tabel1" ref="A4:J9" totalsRowShown="0" headerRowDxfId="21" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}" name="Tabel1" displayName="Tabel1" ref="A4:J9" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A4:J9" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}"/>
   <tableColumns count="10">
-    <tableColumn id="11" xr3:uid="{60446FA3-5B20-442C-B6A4-8EFCA33FCBDA}" name="Belang" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FD154E0F-2AC8-47C8-A1E8-C7BB6A371C52}" name="Formaat" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{F0B04CDC-7073-4197-A4B1-C7C1183C0508}" name="Prioriteit" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{3E48CA4B-7381-4B51-937D-856B47F71F1E}" name="Mijlpaal" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{D3853951-2E2F-4E67-AAAE-47E0C27BC7B9}" name="Beschrijving" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{F5537AA8-5CC1-48F0-8A79-A7F309A087E8}" name="Code part" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{D99FC260-E421-49BC-B32E-D2D8DC52D147}" name="Status" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{14D8C130-60DB-4A29-B889-4978AFAF14D0}" name="Persoon" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{6765A589-0114-41B8-B920-7D21DCC4B9F7}" name="Branch" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{342C098B-23B5-4681-A52B-E16436883EEE}" name="Opmerking" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{60446FA3-5B20-442C-B6A4-8EFCA33FCBDA}" name="Belang" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{FD154E0F-2AC8-47C8-A1E8-C7BB6A371C52}" name="Formaat" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{F0B04CDC-7073-4197-A4B1-C7C1183C0508}" name="Prioriteit" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{3E48CA4B-7381-4B51-937D-856B47F71F1E}" name="Mijlpaal" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{D3853951-2E2F-4E67-AAAE-47E0C27BC7B9}" name="Beschrijving" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{F5537AA8-5CC1-48F0-8A79-A7F309A087E8}" name="Code part" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{D99FC260-E421-49BC-B32E-D2D8DC52D147}" name="Status" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{14D8C130-60DB-4A29-B889-4978AFAF14D0}" name="Persoon" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{6765A589-0114-41B8-B920-7D21DCC4B9F7}" name="Branch" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{342C098B-23B5-4681-A52B-E16436883EEE}" name="Opmerking" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1057,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A647D6D8-2B75-49BC-A998-EBD3E5FC05BB}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
@@ -1147,8 +1156,12 @@
       <c r="E6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="H6" s="3" t="s">
         <v>32</v>
       </c>
@@ -1168,6 +1181,24 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1181,19 +1212,19 @@
           <x14:formula1>
             <xm:f>Lijsten!$C$3:$C$6</xm:f>
           </x14:formula1>
-          <xm:sqref>A4:A7</xm:sqref>
+          <xm:sqref>A4:A8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{514BCFB8-EA50-44F4-B200-DE0889951621}">
           <x14:formula1>
             <xm:f>Lijsten!$E$3:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B4:B7</xm:sqref>
+          <xm:sqref>B4:B8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A109FC9E-2AC9-46D5-9766-88C3F20D5185}">
           <x14:formula1>
             <xm:f>Lijsten!$G$3:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E4:E7</xm:sqref>
+          <xm:sqref>E4:E8</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Added 2 punten (sander)
</commit_message>
<xml_diff>
--- a/TODO.xlsx
+++ b/TODO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsrlnl-my.sharepoint.com/personal/s_kapinga_wsrl_nl/Documents/Documenten/Github/GeoProb-Pipe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6BB675-1AB6-4B37-A836-CEA805BD88A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{7D6BB675-1AB6-4B37-A836-CEA805BD88A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FBDE386-EA7D-4B62-AE5D-1D9B499991B4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{453B4A97-9B0D-4640-BCE1-44769073F81C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{453B4A97-9B0D-4640-BCE1-44769073F81C}"/>
   </bookViews>
   <sheets>
     <sheet name="Lijsten" sheetId="1" state="hidden" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="54">
   <si>
     <t>Belang</t>
   </si>
@@ -195,6 +195,12 @@
   </si>
   <si>
     <t xml:space="preserve">In de onderstaande lijst zijn globale mijlpalen toegevoegd. Dit zijn niet taken, maar punten op de horizon. </t>
+  </si>
+  <si>
+    <t>Controle op som van scenariokansen per uittredepunt. Als de som niet gelijk aan 1,0  dan een warning loggen (Sander)</t>
+  </si>
+  <si>
+    <t>Met model 4a worden is de weerstand van het achterland afhankelijk van maaiveldniveau van het vak en de top van het zand van het ondergrondscenario. Een dikke deklaag heeft meer weerstand dan een dunne. Dit werkt nu ook in de huidige tool. Implementatie bespreken (Sander)</t>
   </si>
 </sst>
 </file>
@@ -254,12 +260,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -267,6 +276,90 @@
   <dxfs count="22">
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -313,62 +406,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -419,6 +456,76 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -437,123 +544,25 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -611,36 +620,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}" name="Tabel13" displayName="Tabel13" ref="A3:H7" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}" name="Tabel13" displayName="Tabel13" ref="A3:H7" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
   <autoFilter ref="A3:H7" xr:uid="{DD17E2B7-5988-4D33-A53A-0233940CAA1F}"/>
   <tableColumns count="8">
-    <tableColumn id="11" xr3:uid="{03EDA042-17EA-4CE6-B062-BCF9D6DC876F}" name="Belang" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{463702E7-7165-4523-9D6B-7ACDA80B9EBD}" name="Prioriteit" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{54B6E275-8C75-4272-90E9-4F6FAD3E0236}" name="Naam" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{49D3B12A-D2A9-4E25-B74D-6BCBEBD88EFA}" name="Beschrijving" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{8FD3869D-6875-466A-8DF3-E625CE109EA2}" name="Application part" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{D973CD04-220F-4A8C-9BF5-59F7D87A76C1}" name="Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{C850139A-3749-435E-9416-B011E18BC87E}" name="Persoon" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{10DD826D-3BF7-4FA1-95A9-305EEE094144}" name="Opmerking" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{03EDA042-17EA-4CE6-B062-BCF9D6DC876F}" name="Belang" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{463702E7-7165-4523-9D6B-7ACDA80B9EBD}" name="Prioriteit" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{54B6E275-8C75-4272-90E9-4F6FAD3E0236}" name="Naam" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{49D3B12A-D2A9-4E25-B74D-6BCBEBD88EFA}" name="Beschrijving" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{8FD3869D-6875-466A-8DF3-E625CE109EA2}" name="Application part" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{D973CD04-220F-4A8C-9BF5-59F7D87A76C1}" name="Status" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{C850139A-3749-435E-9416-B011E18BC87E}" name="Persoon" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{10DD826D-3BF7-4FA1-95A9-305EEE094144}" name="Opmerking" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}" name="Tabel1" displayName="Tabel1" ref="A4:J9" totalsRowShown="0" headerRowDxfId="21" dataDxfId="12">
-  <autoFilter ref="A4:J9" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}" name="Tabel1" displayName="Tabel1" ref="A4:J11" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A4:J11" xr:uid="{8CAEE4E8-642B-4B28-87C3-2C66CFAD0E85}"/>
   <tableColumns count="10">
-    <tableColumn id="11" xr3:uid="{60446FA3-5B20-442C-B6A4-8EFCA33FCBDA}" name="Belang" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FD154E0F-2AC8-47C8-A1E8-C7BB6A371C52}" name="Formaat" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{F0B04CDC-7073-4197-A4B1-C7C1183C0508}" name="Prioriteit" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{3E48CA4B-7381-4B51-937D-856B47F71F1E}" name="Mijlpaal" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{D3853951-2E2F-4E67-AAAE-47E0C27BC7B9}" name="Beschrijving" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{F5537AA8-5CC1-48F0-8A79-A7F309A087E8}" name="Code part" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{D99FC260-E421-49BC-B32E-D2D8DC52D147}" name="Status" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{14D8C130-60DB-4A29-B889-4978AFAF14D0}" name="Persoon" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{6765A589-0114-41B8-B920-7D21DCC4B9F7}" name="Branch" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{342C098B-23B5-4681-A52B-E16436883EEE}" name="Opmerking" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{60446FA3-5B20-442C-B6A4-8EFCA33FCBDA}" name="Belang" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{FD154E0F-2AC8-47C8-A1E8-C7BB6A371C52}" name="Formaat" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{F0B04CDC-7073-4197-A4B1-C7C1183C0508}" name="Prioriteit" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{3E48CA4B-7381-4B51-937D-856B47F71F1E}" name="Mijlpaal" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{D3853951-2E2F-4E67-AAAE-47E0C27BC7B9}" name="Beschrijving" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{F5537AA8-5CC1-48F0-8A79-A7F309A087E8}" name="Code part" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{D99FC260-E421-49BC-B32E-D2D8DC52D147}" name="Status" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{14D8C130-60DB-4A29-B889-4978AFAF14D0}" name="Persoon" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{6765A589-0114-41B8-B920-7D21DCC4B9F7}" name="Branch" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{342C098B-23B5-4681-A52B-E16436883EEE}" name="Opmerking" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -964,14 +973,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{882C4D68-017A-4699-939F-8A0E3184D8BB}">
   <dimension ref="C2:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -988,7 +997,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>1</v>
       </c>
@@ -1005,7 +1014,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>2</v>
       </c>
@@ -1022,7 +1031,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>3</v>
       </c>
@@ -1039,7 +1048,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>4</v>
       </c>
@@ -1058,24 +1067,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A647D6D8-2B75-49BC-A998-EBD3E5FC05BB}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="49.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="34.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1110,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -1117,7 +1126,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -1133,7 +1142,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
         <v>30</v>
@@ -1153,7 +1162,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3" t="s">
         <v>40</v>
@@ -1203,38 +1212,38 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{708ADBE1-0D9E-4DE0-9AAA-27C5B7AA8769}">
-  <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" customWidth="1"/>
-    <col min="5" max="5" width="58.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="58.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D3" s="4" t="s">
         <v>45</v>
       </c>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1266,7 +1275,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1290,7 +1299,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1316,7 +1325,7 @@
       </c>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -1342,7 +1351,7 @@
       </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -1368,7 +1377,7 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1393,6 +1402,46 @@
         <v>39</v>
       </c>
       <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" ht="64.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1406,31 +1455,31 @@
           <x14:formula1>
             <xm:f>Lijsten!$C$3:$C$6</xm:f>
           </x14:formula1>
-          <xm:sqref>A5:A9</xm:sqref>
+          <xm:sqref>A5:A11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AF7C1223-1F19-43C7-AEA8-4005AE0773BC}">
           <x14:formula1>
             <xm:f>Lijsten!$F$3:$F$6</xm:f>
           </x14:formula1>
-          <xm:sqref>G5:G9</xm:sqref>
+          <xm:sqref>G5:G11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{583B3ACE-A229-4F75-8633-D90FF5D192F0}">
           <x14:formula1>
             <xm:f>Lijsten!$E$3:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>C5:C9</xm:sqref>
+          <xm:sqref>C5:C11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{62C78DFC-894B-49C1-8714-567392665842}">
           <x14:formula1>
             <xm:f>Lijsten!$D$3:$D$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B9</xm:sqref>
+          <xm:sqref>B5:B11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{501E8654-1817-4EE0-8353-CA441087B7A7}">
           <x14:formula1>
             <xm:f>Mijlpalen!$C$4:$C$7</xm:f>
           </x14:formula1>
-          <xm:sqref>D5:D9</xm:sqref>
+          <xm:sqref>D5:D11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1441,7 +1490,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AE609A2-61FC-42DC-87CA-5B202EC356A4}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>